<commit_message>
Ship the three-winding case file the Appendix used
</commit_message>
<xml_diff>
--- a/grids/pandapower_3w.xlsx
+++ b/grids/pandapower_3w.xlsx
@@ -1260,7 +1260,7 @@
         <v>1</v>
       </c>
       <c r="D2" s="16" t="n">
-        <v>0.975</v>
+        <v>0.98</v>
       </c>
       <c r="E2" s="16" t="n">
         <v>1.02</v>
@@ -4804,11 +4804,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F8"/>
+  <dimension ref="A1:H8"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.5703125" defaultRowHeight="18"/>
   <cols>
-    <col width="14.85546875" bestFit="1" customWidth="1" style="15" min="2" max="2"/>
-    <col width="14.5703125" bestFit="1" customWidth="1" style="15" min="5" max="5"/>
+    <col width="14.85546875" bestFit="1" customWidth="1" style="15" min="2" max="4"/>
+    <col width="14.5703125" bestFit="1" customWidth="1" style="15" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1" ht="19" customFormat="1" customHeight="1" s="1">
@@ -4819,25 +4819,35 @@
       </c>
       <c r="B1" s="3" t="inlineStr">
         <is>
-          <t>Nominal Current</t>
-        </is>
-      </c>
-      <c r="C1" s="4" t="inlineStr">
+          <t>Z_p</t>
+        </is>
+      </c>
+      <c r="C1" s="3" t="inlineStr">
+        <is>
+          <t>I_p</t>
+        </is>
+      </c>
+      <c r="D1" s="3" t="inlineStr">
+        <is>
+          <t>P_p</t>
+        </is>
+      </c>
+      <c r="E1" s="4" t="inlineStr">
         <is>
           <t>V0 [pu]</t>
         </is>
       </c>
-      <c r="D1" s="4" t="inlineStr">
+      <c r="F1" s="4" t="inlineStr">
         <is>
           <t>V_base [V]</t>
         </is>
       </c>
-      <c r="E1" s="3" t="inlineStr">
+      <c r="G1" s="3" t="inlineStr">
         <is>
           <t>VM min [pu]</t>
         </is>
       </c>
-      <c r="F1" s="3" t="inlineStr">
+      <c r="H1" s="3" t="inlineStr">
         <is>
           <t>VM max [pu]</t>
         </is>
@@ -4851,15 +4861,21 @@
         <v>0</v>
       </c>
       <c r="C2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E2" t="n">
+        <v>1</v>
+      </c>
+      <c r="F2" t="n">
         <v>750</v>
       </c>
-      <c r="E2" t="n">
+      <c r="G2" t="n">
         <v>0.9</v>
       </c>
-      <c r="F2" t="n">
+      <c r="H2" t="n">
         <v>1.1</v>
       </c>
     </row>
@@ -4871,15 +4887,21 @@
         <v>0</v>
       </c>
       <c r="C3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E3" t="n">
+        <v>1</v>
+      </c>
+      <c r="F3" t="n">
         <v>750</v>
       </c>
-      <c r="E3" t="n">
+      <c r="G3" t="n">
         <v>0.9</v>
       </c>
-      <c r="F3" t="n">
+      <c r="H3" t="n">
         <v>1.1</v>
       </c>
     </row>
@@ -4891,15 +4913,21 @@
         <v>0</v>
       </c>
       <c r="C4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D4" t="n">
+        <v>1</v>
+      </c>
+      <c r="E4" t="n">
+        <v>1</v>
+      </c>
+      <c r="F4" t="n">
         <v>750</v>
       </c>
-      <c r="E4" t="n">
+      <c r="G4" t="n">
         <v>0.9</v>
       </c>
-      <c r="F4" t="n">
+      <c r="H4" t="n">
         <v>1.1</v>
       </c>
     </row>
@@ -4911,15 +4939,21 @@
         <v>0</v>
       </c>
       <c r="C5" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D5" t="n">
+        <v>1</v>
+      </c>
+      <c r="E5" t="n">
+        <v>1</v>
+      </c>
+      <c r="F5" t="n">
         <v>750</v>
       </c>
-      <c r="E5" t="n">
+      <c r="G5" t="n">
         <v>0.9</v>
       </c>
-      <c r="F5" t="n">
+      <c r="H5" t="n">
         <v>1.1</v>
       </c>
     </row>
@@ -4931,15 +4965,21 @@
         <v>0</v>
       </c>
       <c r="C6" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D6" t="n">
+        <v>1</v>
+      </c>
+      <c r="E6" t="n">
+        <v>1</v>
+      </c>
+      <c r="F6" t="n">
         <v>750</v>
       </c>
-      <c r="E6" t="n">
+      <c r="G6" t="n">
         <v>0.9</v>
       </c>
-      <c r="F6" t="n">
+      <c r="H6" t="n">
         <v>1.1</v>
       </c>
     </row>
@@ -4951,15 +4991,21 @@
         <v>0</v>
       </c>
       <c r="C7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D7" t="n">
+        <v>1</v>
+      </c>
+      <c r="E7" t="n">
+        <v>1</v>
+      </c>
+      <c r="F7" t="n">
         <v>750</v>
       </c>
-      <c r="E7" t="n">
+      <c r="G7" t="n">
         <v>0.9</v>
       </c>
-      <c r="F7" t="n">
+      <c r="H7" t="n">
         <v>1.1</v>
       </c>
     </row>
@@ -4971,15 +5017,21 @@
         <v>0</v>
       </c>
       <c r="C8" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D8" t="n">
+        <v>1</v>
+      </c>
+      <c r="E8" t="n">
+        <v>1</v>
+      </c>
+      <c r="F8" t="n">
         <v>750</v>
       </c>
-      <c r="E8" t="n">
+      <c r="G8" t="n">
         <v>0.9</v>
       </c>
-      <c r="F8" t="n">
+      <c r="H8" t="n">
         <v>1.1</v>
       </c>
     </row>

</xml_diff>